<commit_message>
Fix generation of purchaser price emission factors for years 2014, 2015 and 2016.
</commit_message>
<xml_diff>
--- a/doc/OpenIO-Canada-classification-structure.xlsx
+++ b/doc/OpenIO-Canada-classification-structure.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\11max\PycharmProjects\OpenIOCanada\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECEFC903-24A6-4B44-9E69-11D4B7C52911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CB53C2-23F4-46D0-B1BB-E903A768DD47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6D781A35-9AD2-44F9-90F7-44301FF10485}"/>
   </bookViews>
@@ -48765,231 +48765,231 @@
       </c>
     </row>
     <row r="1960" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C1960" t="s">
-        <v>2934</v>
+      <c r="A1960" t="s">
+        <v>568</v>
+      </c>
+      <c r="B1960" t="s">
+        <v>4936</v>
       </c>
     </row>
     <row r="1961" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C1961" t="s">
-        <v>2935</v>
+        <v>2927</v>
       </c>
     </row>
     <row r="1962" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C1962" t="s">
-        <v>2936</v>
+        <v>2928</v>
       </c>
     </row>
     <row r="1963" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1963" t="s">
-        <v>568</v>
-      </c>
-      <c r="B1963" t="s">
-        <v>4936</v>
+      <c r="C1963" t="s">
+        <v>2929</v>
       </c>
     </row>
     <row r="1964" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C1964" t="s">
-        <v>2927</v>
+        <v>2930</v>
       </c>
     </row>
     <row r="1965" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C1965" t="s">
-        <v>2928</v>
+        <v>2931</v>
       </c>
     </row>
     <row r="1966" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C1966" t="s">
-        <v>2929</v>
+        <v>2932</v>
       </c>
     </row>
     <row r="1967" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C1967" t="s">
-        <v>2930</v>
+        <v>2933</v>
       </c>
     </row>
     <row r="1968" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C1968" t="s">
-        <v>2931</v>
+      <c r="A1968" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1968" t="s">
+        <v>571</v>
       </c>
     </row>
     <row r="1969" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1969" t="s">
-        <v>2932</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="1970" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1970" t="s">
-        <v>2933</v>
+        <v>2918</v>
       </c>
     </row>
     <row r="1971" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1971" t="s">
-        <v>570</v>
-      </c>
-      <c r="B1971" t="s">
-        <v>571</v>
+      <c r="C1971" t="s">
+        <v>2919</v>
       </c>
     </row>
     <row r="1972" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1972" t="s">
-        <v>2917</v>
+        <v>2920</v>
       </c>
     </row>
     <row r="1973" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C1973" t="s">
-        <v>2918</v>
+      <c r="A1973" t="s">
+        <v>572</v>
+      </c>
+      <c r="B1973" t="s">
+        <v>573</v>
       </c>
     </row>
     <row r="1974" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1974" t="s">
-        <v>2919</v>
+        <v>2921</v>
       </c>
     </row>
     <row r="1975" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1975" t="s">
-        <v>2920</v>
+        <v>2922</v>
       </c>
     </row>
     <row r="1976" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1976" t="s">
-        <v>572</v>
-      </c>
-      <c r="B1976" t="s">
-        <v>573</v>
+      <c r="C1976" t="s">
+        <v>2923</v>
       </c>
     </row>
     <row r="1977" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1977" t="s">
-        <v>2921</v>
+        <v>2924</v>
       </c>
     </row>
     <row r="1978" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1978" t="s">
-        <v>2922</v>
+        <v>2925</v>
       </c>
     </row>
     <row r="1979" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1979" t="s">
-        <v>2923</v>
+        <v>2926</v>
       </c>
     </row>
     <row r="1980" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C1980" t="s">
-        <v>2924</v>
+      <c r="A1980" t="s">
+        <v>574</v>
+      </c>
+      <c r="B1980" t="s">
+        <v>575</v>
       </c>
     </row>
     <row r="1981" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1981" t="s">
-        <v>2925</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="1982" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1982" t="s">
-        <v>2926</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="1983" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1983" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="B1983" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="1984" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1984" t="s">
-        <v>2915</v>
+        <v>2912</v>
       </c>
     </row>
     <row r="1985" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1985" t="s">
-        <v>2916</v>
+        <v>2913</v>
       </c>
     </row>
     <row r="1986" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1986" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B1986" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="1987" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1987" t="s">
-        <v>2912</v>
+        <v>2914</v>
       </c>
     </row>
     <row r="1988" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1988" t="s">
-        <v>2913</v>
+        <v>2937</v>
       </c>
     </row>
     <row r="1989" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1989" t="s">
-        <v>578</v>
-      </c>
-      <c r="B1989" t="s">
-        <v>579</v>
+      <c r="C1989" t="s">
+        <v>2938</v>
       </c>
     </row>
     <row r="1990" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1990" t="s">
-        <v>2914</v>
+        <v>2939</v>
       </c>
     </row>
     <row r="1991" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1991" t="s">
-        <v>2937</v>
+        <v>2940</v>
       </c>
     </row>
     <row r="1992" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1992" t="s">
-        <v>2938</v>
+        <v>2941</v>
       </c>
     </row>
     <row r="1993" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1993" t="s">
-        <v>2939</v>
+        <v>2942</v>
       </c>
     </row>
     <row r="1994" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1994" t="s">
-        <v>2940</v>
+        <v>2943</v>
       </c>
     </row>
     <row r="1995" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1995" t="s">
-        <v>2941</v>
+        <v>2944</v>
       </c>
     </row>
     <row r="1996" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1996" t="s">
-        <v>2942</v>
+        <v>2945</v>
       </c>
     </row>
     <row r="1997" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1997" t="s">
-        <v>2943</v>
+        <v>2946</v>
       </c>
     </row>
     <row r="1998" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1998" t="s">
-        <v>2944</v>
+        <v>2947</v>
       </c>
     </row>
     <row r="1999" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C1999" t="s">
-        <v>2945</v>
+        <v>2934</v>
       </c>
     </row>
     <row r="2000" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C2000" t="s">
-        <v>2946</v>
+        <v>2935</v>
       </c>
     </row>
     <row r="2001" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C2001" t="s">
-        <v>2947</v>
+        <v>2936</v>
       </c>
     </row>
     <row r="2002" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>